<commit_message>
feat: publish qualified DealBench 1.1 task source
</commit_message>
<xml_diff>
--- a/benchmark/dealbench100/release/assets/project-canopy/10-debt-schedule.xlsx
+++ b/benchmark/dealbench100/release/assets/project-canopy/10-debt-schedule.xlsx
@@ -13,17 +13,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Instrument</t>
+          <t>Instrument / constraint</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Balance ($m)</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rate</t>
+          <t>Unit</t>
         </is>
       </c>
     </row>
@@ -36,8 +36,10 @@
       <c r="B2">
         <v>108.72</v>
       </c>
-      <c r="C2">
-        <v>0.071</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -49,8 +51,10 @@
       <c r="B3">
         <v>42.28</v>
       </c>
-      <c r="C3">
-        <v>0.082</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -62,8 +66,55 @@
       <c r="B4">
         <v>20.0</v>
       </c>
-      <c r="C4">
-        <v>0.0</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Maximum entry leverage</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>5.0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>x EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Exit multiple</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>8.8</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>x EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Approved five-year sponsor IRR floor</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>20.0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: publish qualified DealBench 1.1 task source (#1)
</commit_message>
<xml_diff>
--- a/benchmark/dealbench100/release/assets/project-canopy/10-debt-schedule.xlsx
+++ b/benchmark/dealbench100/release/assets/project-canopy/10-debt-schedule.xlsx
@@ -13,17 +13,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Instrument</t>
+          <t>Instrument / constraint</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Balance ($m)</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Rate</t>
+          <t>Unit</t>
         </is>
       </c>
     </row>
@@ -36,8 +36,10 @@
       <c r="B2">
         <v>108.72</v>
       </c>
-      <c r="C2">
-        <v>0.071</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -49,8 +51,10 @@
       <c r="B3">
         <v>42.28</v>
       </c>
-      <c r="C3">
-        <v>0.082</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -62,8 +66,55 @@
       <c r="B4">
         <v>20.0</v>
       </c>
-      <c r="C4">
-        <v>0.0</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USD m</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Maximum entry leverage</t>
+        </is>
+      </c>
+      <c r="B5">
+        <v>5.0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>x EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Exit multiple</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>8.8</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>x EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Approved five-year sponsor IRR floor</t>
+        </is>
+      </c>
+      <c r="B7">
+        <v>20.0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>